<commit_message>
Direct Write Excel for Crane no.1 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.1.xlsx
+++ b/FM-MN-07_Crane no.1.xlsx
@@ -1759,7 +1759,11 @@
       <c r="E6" s="13" t="inlineStr"/>
       <c r="F6" s="13" t="inlineStr"/>
       <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="13" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="13" t="inlineStr"/>
       <c r="J6" s="13" t="inlineStr"/>
       <c r="K6" s="13" t="inlineStr"/>
@@ -1800,7 +1804,11 @@
       <c r="E7" s="13" t="inlineStr"/>
       <c r="F7" s="13" t="inlineStr"/>
       <c r="G7" s="13" t="inlineStr"/>
-      <c r="H7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="13" t="inlineStr"/>
       <c r="J7" s="13" t="inlineStr"/>
       <c r="K7" s="13" t="inlineStr"/>
@@ -1842,7 +1850,11 @@
       <c r="E8" s="13" t="inlineStr"/>
       <c r="F8" s="13" t="inlineStr"/>
       <c r="G8" s="13" t="inlineStr"/>
-      <c r="H8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="13" t="inlineStr"/>
       <c r="J8" s="13" t="inlineStr"/>
       <c r="K8" s="13" t="inlineStr"/>
@@ -1883,7 +1895,11 @@
       <c r="E9" s="13" t="inlineStr"/>
       <c r="F9" s="13" t="inlineStr"/>
       <c r="G9" s="13" t="inlineStr"/>
-      <c r="H9" s="13" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="13" t="inlineStr"/>
       <c r="J9" s="13" t="inlineStr"/>
       <c r="K9" s="13" t="inlineStr"/>
@@ -1925,7 +1941,11 @@
       <c r="E10" s="13" t="inlineStr"/>
       <c r="F10" s="13" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="13" t="inlineStr"/>
       <c r="J10" s="13" t="inlineStr"/>
       <c r="K10" s="13" t="inlineStr"/>
@@ -1966,7 +1986,11 @@
       <c r="E11" s="13" t="inlineStr"/>
       <c r="F11" s="13" t="inlineStr"/>
       <c r="G11" s="13" t="inlineStr"/>
-      <c r="H11" s="13" t="inlineStr"/>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I11" s="13" t="inlineStr"/>
       <c r="J11" s="13" t="inlineStr"/>
       <c r="K11" s="13" t="inlineStr"/>
@@ -2069,7 +2093,11 @@
       <c r="E14" s="30" t="inlineStr"/>
       <c r="F14" s="30" t="inlineStr"/>
       <c r="G14" s="30" t="inlineStr"/>
-      <c r="H14" s="30" t="inlineStr"/>
+      <c r="H14" s="35" t="inlineStr">
+        <is>
+          <t>นายอดุลย์  ศิริรัตน์</t>
+        </is>
+      </c>
       <c r="I14" s="30" t="inlineStr"/>
       <c r="J14" s="30" t="inlineStr"/>
       <c r="K14" s="30" t="inlineStr"/>
@@ -2206,7 +2234,11 @@
       </c>
     </row>
     <row r="19" ht="342.75" customHeight="1">
-      <c r="B19" s="44" t="inlineStr"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="23.25" customHeight="1"/>
     <row r="21" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Safe Direct Write Excel for Crane no.1 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.1.xlsx
+++ b/FM-MN-07_Crane no.1.xlsx
@@ -1764,7 +1764,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="13" t="inlineStr"/>
       <c r="K6" s="13" t="inlineStr"/>
       <c r="L6" s="13" t="inlineStr"/>
@@ -1809,7 +1813,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="13" t="inlineStr"/>
       <c r="K7" s="13" t="inlineStr"/>
       <c r="L7" s="13" t="inlineStr"/>
@@ -1855,7 +1863,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="13" t="inlineStr"/>
       <c r="K8" s="13" t="inlineStr"/>
       <c r="L8" s="13" t="inlineStr"/>
@@ -1900,7 +1912,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="13" t="inlineStr"/>
       <c r="K9" s="13" t="inlineStr"/>
       <c r="L9" s="13" t="inlineStr"/>
@@ -1946,7 +1962,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="13" t="inlineStr"/>
       <c r="K10" s="13" t="inlineStr"/>
       <c r="L10" s="13" t="inlineStr"/>
@@ -1991,7 +2011,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J11" s="13" t="inlineStr"/>
       <c r="K11" s="13" t="inlineStr"/>
       <c r="L11" s="13" t="inlineStr"/>
@@ -2098,7 +2122,11 @@
           <t>นายอดุลย์  ศิริรัตน์</t>
         </is>
       </c>
-      <c r="I14" s="30" t="inlineStr"/>
+      <c r="I14" s="35" t="inlineStr">
+        <is>
+          <t>นายอดุลย์  ศิริรัตน์</t>
+        </is>
+      </c>
       <c r="J14" s="30" t="inlineStr"/>
       <c r="K14" s="30" t="inlineStr"/>
       <c r="L14" s="30" t="inlineStr"/>
@@ -2236,7 +2264,7 @@
     <row r="19" ht="342.75" customHeight="1">
       <c r="B19" s="44" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
+          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 7]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for Crane no.1 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.1.xlsx
+++ b/FM-MN-07_Crane no.1.xlsx
@@ -1769,7 +1769,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="13" t="inlineStr"/>
       <c r="L6" s="13" t="inlineStr"/>
       <c r="M6" s="13" t="inlineStr"/>
@@ -1818,7 +1822,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="13" t="inlineStr"/>
       <c r="L7" s="13" t="inlineStr"/>
       <c r="M7" s="13" t="inlineStr"/>
@@ -1868,7 +1876,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="13" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="13" t="inlineStr"/>
       <c r="L8" s="13" t="inlineStr"/>
       <c r="M8" s="13" t="inlineStr"/>
@@ -1917,7 +1929,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="13" t="inlineStr"/>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="13" t="inlineStr"/>
       <c r="L9" s="13" t="inlineStr"/>
       <c r="M9" s="13" t="inlineStr"/>
@@ -1967,7 +1983,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr"/>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="13" t="inlineStr"/>
       <c r="L10" s="13" t="inlineStr"/>
       <c r="M10" s="13" t="inlineStr"/>
@@ -2016,7 +2036,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr"/>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K11" s="13" t="inlineStr"/>
       <c r="L11" s="13" t="inlineStr"/>
       <c r="M11" s="13" t="inlineStr"/>
@@ -2127,7 +2151,11 @@
           <t>นายอดุลย์  ศิริรัตน์</t>
         </is>
       </c>
-      <c r="J14" s="30" t="inlineStr"/>
+      <c r="J14" s="35" t="inlineStr">
+        <is>
+          <t>นายอดุลย์  ศิริรัตน์</t>
+        </is>
+      </c>
       <c r="K14" s="30" t="inlineStr"/>
       <c r="L14" s="30" t="inlineStr"/>
       <c r="M14" s="30" t="inlineStr"/>
@@ -2264,7 +2292,7 @@
     <row r="19" ht="342.75" customHeight="1">
       <c r="B19" s="44" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 7]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
+          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 7]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 8]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for Crane no.1 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_Crane no.1.xlsx
+++ b/FM-MN-07_Crane no.1.xlsx
@@ -1775,7 +1775,11 @@
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr"/>
-      <c r="L6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="13" t="inlineStr"/>
       <c r="N6" s="13" t="inlineStr"/>
       <c r="O6" s="13" t="inlineStr"/>
@@ -1828,7 +1832,11 @@
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr"/>
-      <c r="L7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="13" t="inlineStr"/>
       <c r="N7" s="13" t="inlineStr"/>
       <c r="O7" s="13" t="inlineStr"/>
@@ -1882,7 +1890,11 @@
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr"/>
-      <c r="L8" s="13" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="13" t="inlineStr"/>
       <c r="N8" s="13" t="inlineStr"/>
       <c r="O8" s="13" t="inlineStr"/>
@@ -1935,7 +1947,11 @@
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr"/>
-      <c r="L9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="13" t="inlineStr"/>
       <c r="N9" s="13" t="inlineStr"/>
       <c r="O9" s="13" t="inlineStr"/>
@@ -1989,7 +2005,11 @@
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr"/>
-      <c r="L10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="13" t="inlineStr"/>
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="13" t="inlineStr"/>
@@ -2042,7 +2062,11 @@
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr"/>
-      <c r="L11" s="13" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M11" s="13" t="inlineStr"/>
       <c r="N11" s="13" t="inlineStr"/>
       <c r="O11" s="13" t="inlineStr"/>
@@ -2157,7 +2181,11 @@
         </is>
       </c>
       <c r="K14" s="30" t="inlineStr"/>
-      <c r="L14" s="30" t="inlineStr"/>
+      <c r="L14" s="35" t="inlineStr">
+        <is>
+          <t>นายอดุลย์  ศิริรัตน์</t>
+        </is>
+      </c>
       <c r="M14" s="30" t="inlineStr"/>
       <c r="N14" s="30" t="inlineStr"/>
       <c r="O14" s="30" t="inlineStr"/>
@@ -2292,7 +2320,7 @@
     <row r="19" ht="342.75" customHeight="1">
       <c r="B19" s="44" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 7]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 8]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
+          <t>[วันที่ 6]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 7]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 8]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด,  [วันที่ 10]: ข้อ 3: สายสลิงเครนตัวเล็กมีการบิดงอ, ข้อ 6: เสียงสัญญาณเตือนไม่ดังมีแค่สัญญาณไฟและเครนตัวเล็กมีเสียงดังเวลากดขึ้นสุด</t>
         </is>
       </c>
     </row>

</xml_diff>